<commit_message>
New filesi n uploaded files
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_Sample_Errors_1.xlsx
+++ b/IEF_Home/UploadedFiles/3_LT_Vehicles_LIST_Sample_Errors_1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20415"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D431FA76-8EC1-4E17-B383-C373712D8B1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A50C4A4-18C9-4053-B51C-81B880A83607}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1140" windowWidth="20418" windowHeight="13440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="204">
   <si>
     <t>Format_Version</t>
   </si>
@@ -313,9 +313,6 @@
   </si>
   <si>
     <t>dataset_conversion_info</t>
-  </si>
-  <si>
-    <t>Numbers manually copied from original source (pdf) to Excel spreadsheet</t>
   </si>
   <si>
     <t>review_date</t>
@@ -1138,6 +1135,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="15" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1164,21 +1176,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1537,18 +1534,18 @@
       <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:11" ht="15.6">
-      <c r="B2" s="67" t="s">
+      <c r="B2" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="74"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="67" t="s">
+      <c r="F2" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="69"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="74"/>
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11">
@@ -1566,7 +1563,7 @@
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="75" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="10" t="s">
@@ -1576,7 +1573,7 @@
         <v>28</v>
       </c>
       <c r="E4" s="51" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F4" s="43" t="s">
         <v>30</v>
@@ -1590,15 +1587,15 @@
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="71"/>
+      <c r="B5" s="76"/>
       <c r="C5" s="14" t="s">
         <v>31</v>
       </c>
       <c r="D5" s="54" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E5" s="51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F5" s="52" t="s">
         <v>29</v>
@@ -1618,7 +1615,7 @@
         <v>21</v>
       </c>
       <c r="E6" s="51" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F6" s="44" t="s">
         <v>0</v>
@@ -1634,7 +1631,7 @@
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" s="72" t="s">
+      <c r="B7" s="77" t="s">
         <v>34</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -1644,7 +1641,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="51" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F7" s="44" t="s">
         <v>1</v>
@@ -1653,7 +1650,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="64" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I7" s="20"/>
       <c r="J7" s="1" t="s">
@@ -1665,7 +1662,7 @@
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8" s="72"/>
+      <c r="B8" s="77"/>
       <c r="C8" s="14" t="s">
         <v>36</v>
       </c>
@@ -1673,7 +1670,7 @@
         <v>3</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F8" s="44" t="s">
         <v>6</v>
@@ -1689,15 +1686,15 @@
       <c r="A9">
         <v>6</v>
       </c>
-      <c r="B9" s="72"/>
+      <c r="B9" s="77"/>
       <c r="C9" s="14" t="s">
         <v>37</v>
       </c>
       <c r="D9" s="55" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E9" s="51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F9" s="44" t="s">
         <v>7</v>
@@ -1713,15 +1710,15 @@
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="B10" s="72"/>
+      <c r="B10" s="77"/>
       <c r="C10" s="14" t="s">
         <v>38</v>
       </c>
       <c r="D10" s="55" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E10" s="51" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F10" s="46" t="s">
         <v>2</v>
@@ -1730,7 +1727,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I10" s="36">
         <v>20</v>
@@ -1741,23 +1738,23 @@
       <c r="A11">
         <v>8</v>
       </c>
-      <c r="B11" s="73" t="s">
+      <c r="B11" s="78" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="33" t="s">
         <v>40</v>
       </c>
       <c r="D11" s="54" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H11" s="48" t="s">
         <v>8</v>
@@ -1774,15 +1771,15 @@
       <c r="A12">
         <v>9</v>
       </c>
-      <c r="B12" s="74"/>
+      <c r="B12" s="79"/>
       <c r="C12" s="33" t="s">
         <v>41</v>
       </c>
       <c r="D12" s="54" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E12" s="51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F12" s="25" t="s">
         <v>14</v>
@@ -1794,7 +1791,7 @@
         <v>16</v>
       </c>
       <c r="I12" s="66" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>29</v>
@@ -1805,15 +1802,15 @@
       <c r="A13">
         <v>10</v>
       </c>
-      <c r="B13" s="74"/>
+      <c r="B13" s="79"/>
       <c r="C13" s="33" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D13" s="54" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E13" s="51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F13" s="25" t="s">
         <v>11</v>
@@ -1825,7 +1822,7 @@
         <v>17</v>
       </c>
       <c r="I13" s="66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>29</v>
@@ -1836,15 +1833,15 @@
       <c r="A14">
         <v>11</v>
       </c>
-      <c r="B14" s="74"/>
+      <c r="B14" s="79"/>
       <c r="C14" s="33" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="54" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E14" s="51" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F14" s="26" t="s">
         <v>15</v>
@@ -1856,7 +1853,7 @@
         <v>18</v>
       </c>
       <c r="I14" s="66" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>29</v>
@@ -1867,13 +1864,13 @@
       <c r="A15">
         <v>12</v>
       </c>
-      <c r="B15" s="74"/>
+      <c r="B15" s="79"/>
       <c r="C15" s="33" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="54"/>
       <c r="E15" s="51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F15" s="25" t="s">
         <v>12</v>
@@ -1885,7 +1882,7 @@
         <v>19</v>
       </c>
       <c r="I15" s="66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>29</v>
@@ -1896,7 +1893,7 @@
       <c r="A16">
         <v>13</v>
       </c>
-      <c r="B16" s="74"/>
+      <c r="B16" s="79"/>
       <c r="C16" s="33" t="s">
         <v>44</v>
       </c>
@@ -1904,7 +1901,7 @@
         <v>21</v>
       </c>
       <c r="E16" s="51" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F16" s="52" t="s">
         <v>29</v>
@@ -1914,7 +1911,7 @@
         <v>20</v>
       </c>
       <c r="I16" s="66" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>29</v>
@@ -1925,15 +1922,15 @@
       <c r="A17">
         <v>14</v>
       </c>
-      <c r="B17" s="74"/>
+      <c r="B17" s="79"/>
       <c r="C17" s="33" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="54" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F17" s="52" t="s">
         <v>29</v>
@@ -1946,15 +1943,15 @@
       <c r="A18">
         <v>15</v>
       </c>
-      <c r="B18" s="74"/>
+      <c r="B18" s="79"/>
       <c r="C18" s="33" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="54" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E18" s="51" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F18" s="52" t="s">
         <v>29</v>
@@ -1966,15 +1963,15 @@
       <c r="A19">
         <v>16</v>
       </c>
-      <c r="B19" s="74"/>
+      <c r="B19" s="79"/>
       <c r="C19" s="33" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F19" s="52" t="s">
         <v>29</v>
@@ -1986,15 +1983,15 @@
       <c r="A20">
         <v>17</v>
       </c>
-      <c r="B20" s="74"/>
+      <c r="B20" s="79"/>
       <c r="C20" s="33" t="s">
         <v>48</v>
       </c>
       <c r="D20" s="54" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E20" s="51" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F20" s="52" t="s">
         <v>29</v>
@@ -2006,17 +2003,17 @@
       <c r="A21">
         <v>18</v>
       </c>
-      <c r="B21" s="75" t="s">
+      <c r="B21" s="80" t="s">
         <v>49</v>
       </c>
       <c r="C21" s="33" t="s">
         <v>50</v>
       </c>
       <c r="D21" s="54" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E21" s="51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F21" s="53" t="s">
         <v>29</v>
@@ -2030,15 +2027,15 @@
       <c r="A22">
         <v>19</v>
       </c>
-      <c r="B22" s="75"/>
+      <c r="B22" s="80"/>
       <c r="C22" s="33" t="s">
         <v>51</v>
       </c>
       <c r="D22" s="54" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E22" s="51" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F22" s="62" t="s">
         <v>29</v>
@@ -2049,15 +2046,15 @@
       <c r="A23">
         <v>20</v>
       </c>
-      <c r="B23" s="75"/>
+      <c r="B23" s="80"/>
       <c r="C23" s="33" t="s">
         <v>52</v>
       </c>
       <c r="D23" s="55" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E23" s="51" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F23" s="62" t="s">
         <v>29</v>
@@ -2068,7 +2065,7 @@
       <c r="A24">
         <v>21</v>
       </c>
-      <c r="B24" s="75"/>
+      <c r="B24" s="80"/>
       <c r="C24" s="33" t="s">
         <v>53</v>
       </c>
@@ -2076,7 +2073,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F24" s="62" t="s">
         <v>29</v>
@@ -2088,7 +2085,7 @@
       <c r="A25">
         <v>22</v>
       </c>
-      <c r="B25" s="75"/>
+      <c r="B25" s="80"/>
       <c r="C25" s="33" t="s">
         <v>20</v>
       </c>
@@ -2096,7 +2093,7 @@
         <v>21</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F25" s="62" t="s">
         <v>29</v>
@@ -2108,7 +2105,7 @@
       <c r="A26">
         <v>23</v>
       </c>
-      <c r="B26" s="76" t="s">
+      <c r="B26" s="67" t="s">
         <v>54</v>
       </c>
       <c r="C26" s="41" t="s">
@@ -2118,7 +2115,7 @@
         <v>14</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F26" s="62" t="s">
         <v>29</v>
@@ -2131,7 +2128,7 @@
       <c r="A27">
         <v>24</v>
       </c>
-      <c r="B27" s="76"/>
+      <c r="B27" s="67"/>
       <c r="C27" s="41" t="s">
         <v>56</v>
       </c>
@@ -2139,7 +2136,7 @@
         <v>798</v>
       </c>
       <c r="E27" s="51" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F27" s="62" t="s">
         <v>29</v>
@@ -2151,7 +2148,7 @@
       <c r="A28">
         <v>25</v>
       </c>
-      <c r="B28" s="76"/>
+      <c r="B28" s="67"/>
       <c r="C28" s="41" t="s">
         <v>57</v>
       </c>
@@ -2171,7 +2168,7 @@
       <c r="A29">
         <v>26</v>
       </c>
-      <c r="B29" s="76"/>
+      <c r="B29" s="67"/>
       <c r="C29" s="41" t="s">
         <v>58</v>
       </c>
@@ -2191,7 +2188,7 @@
       <c r="A30">
         <v>27</v>
       </c>
-      <c r="B30" s="76"/>
+      <c r="B30" s="67"/>
       <c r="C30" s="41" t="s">
         <v>59</v>
       </c>
@@ -2211,7 +2208,7 @@
       <c r="A31">
         <v>28</v>
       </c>
-      <c r="B31" s="76"/>
+      <c r="B31" s="67"/>
       <c r="C31" s="41" t="s">
         <v>60</v>
       </c>
@@ -2231,12 +2228,12 @@
       <c r="A32">
         <v>29</v>
       </c>
-      <c r="B32" s="76"/>
+      <c r="B32" s="67"/>
       <c r="C32" s="41" t="s">
         <v>61</v>
       </c>
       <c r="D32" s="57" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E32" s="51" t="s">
         <v>29</v>
@@ -2250,7 +2247,7 @@
       <c r="A33">
         <v>30</v>
       </c>
-      <c r="B33" s="76"/>
+      <c r="B33" s="67"/>
       <c r="C33" s="41" t="s">
         <v>62</v>
       </c>
@@ -2269,7 +2266,7 @@
       <c r="A34">
         <v>31</v>
       </c>
-      <c r="B34" s="76"/>
+      <c r="B34" s="67"/>
       <c r="C34" s="41" t="s">
         <v>63</v>
       </c>
@@ -2288,7 +2285,7 @@
       <c r="A35">
         <v>32</v>
       </c>
-      <c r="B35" s="76"/>
+      <c r="B35" s="67"/>
       <c r="C35" s="31" t="s">
         <v>64</v>
       </c>
@@ -2308,7 +2305,7 @@
       <c r="A36">
         <v>33</v>
       </c>
-      <c r="B36" s="76"/>
+      <c r="B36" s="67"/>
       <c r="C36" s="31" t="s">
         <v>65</v>
       </c>
@@ -2328,7 +2325,7 @@
       <c r="A37">
         <v>34</v>
       </c>
-      <c r="B37" s="76"/>
+      <c r="B37" s="67"/>
       <c r="C37" s="31" t="s">
         <v>66</v>
       </c>
@@ -2347,7 +2344,7 @@
       <c r="A38">
         <v>35</v>
       </c>
-      <c r="B38" s="76"/>
+      <c r="B38" s="67"/>
       <c r="C38" s="31" t="s">
         <v>67</v>
       </c>
@@ -2367,7 +2364,7 @@
       <c r="A39">
         <v>36</v>
       </c>
-      <c r="B39" s="76"/>
+      <c r="B39" s="67"/>
       <c r="C39" s="31" t="s">
         <v>68</v>
       </c>
@@ -2388,7 +2385,7 @@
       <c r="A40">
         <v>37</v>
       </c>
-      <c r="B40" s="76"/>
+      <c r="B40" s="67"/>
       <c r="C40" s="31" t="s">
         <v>69</v>
       </c>
@@ -2410,7 +2407,7 @@
       <c r="A41">
         <v>38</v>
       </c>
-      <c r="B41" s="76"/>
+      <c r="B41" s="67"/>
       <c r="C41" s="31" t="s">
         <v>70</v>
       </c>
@@ -2431,7 +2428,7 @@
       <c r="A42">
         <v>39</v>
       </c>
-      <c r="B42" s="76"/>
+      <c r="B42" s="67"/>
       <c r="C42" s="31" t="s">
         <v>71</v>
       </c>
@@ -2452,7 +2449,7 @@
       <c r="A43">
         <v>40</v>
       </c>
-      <c r="B43" s="76"/>
+      <c r="B43" s="67"/>
       <c r="C43" s="31" t="s">
         <v>72</v>
       </c>
@@ -2474,7 +2471,7 @@
       <c r="A44">
         <v>41</v>
       </c>
-      <c r="B44" s="76"/>
+      <c r="B44" s="67"/>
       <c r="C44" s="31" t="s">
         <v>73</v>
       </c>
@@ -2496,7 +2493,7 @@
       <c r="A45">
         <v>42</v>
       </c>
-      <c r="B45" s="76"/>
+      <c r="B45" s="67"/>
       <c r="C45" s="31" t="s">
         <v>74</v>
       </c>
@@ -2520,7 +2517,7 @@
       <c r="A46">
         <v>43</v>
       </c>
-      <c r="B46" s="76"/>
+      <c r="B46" s="67"/>
       <c r="C46" s="31" t="s">
         <v>75</v>
       </c>
@@ -2543,7 +2540,7 @@
       <c r="A47">
         <v>44</v>
       </c>
-      <c r="B47" s="76"/>
+      <c r="B47" s="67"/>
       <c r="C47" s="31" t="s">
         <v>76</v>
       </c>
@@ -2564,7 +2561,7 @@
       <c r="A48">
         <v>45</v>
       </c>
-      <c r="B48" s="76"/>
+      <c r="B48" s="67"/>
       <c r="C48" s="31" t="s">
         <v>77</v>
       </c>
@@ -2585,7 +2582,7 @@
       <c r="A49">
         <v>46</v>
       </c>
-      <c r="B49" s="76"/>
+      <c r="B49" s="67"/>
       <c r="C49" s="31" t="s">
         <v>78</v>
       </c>
@@ -2608,15 +2605,15 @@
       <c r="A50">
         <v>47</v>
       </c>
-      <c r="B50" s="76"/>
+      <c r="B50" s="67"/>
       <c r="C50" s="23" t="s">
         <v>79</v>
       </c>
       <c r="D50" s="54" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E50" s="51" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F50" s="62" t="s">
         <v>29</v>
@@ -2630,15 +2627,15 @@
       <c r="A51">
         <v>48</v>
       </c>
-      <c r="B51" s="76"/>
+      <c r="B51" s="67"/>
       <c r="C51" s="23" t="s">
         <v>80</v>
       </c>
       <c r="D51" s="54" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E51" s="51" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F51" s="62" t="s">
         <v>29</v>
@@ -2651,15 +2648,15 @@
       <c r="A52">
         <v>49</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="67"/>
       <c r="C52" s="23" t="s">
         <v>81</v>
       </c>
       <c r="D52" s="54" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E52" s="51" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F52" s="62" t="s">
         <v>29</v>
@@ -2673,7 +2670,7 @@
       <c r="A53">
         <v>50</v>
       </c>
-      <c r="B53" s="77" t="s">
+      <c r="B53" s="68" t="s">
         <v>82</v>
       </c>
       <c r="C53" s="14" t="s">
@@ -2683,7 +2680,7 @@
         <v>84</v>
       </c>
       <c r="E53" s="51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F53" s="62" t="s">
         <v>29</v>
@@ -2695,7 +2692,7 @@
       <c r="A54">
         <v>51</v>
       </c>
-      <c r="B54" s="77"/>
+      <c r="B54" s="68"/>
       <c r="C54" s="14" t="s">
         <v>85</v>
       </c>
@@ -2703,7 +2700,7 @@
         <v>86</v>
       </c>
       <c r="E54" s="51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F54" s="62" t="s">
         <v>29</v>
@@ -2715,15 +2712,15 @@
       <c r="A55">
         <v>52</v>
       </c>
-      <c r="B55" s="77"/>
+      <c r="B55" s="68"/>
       <c r="C55" s="14" t="s">
         <v>87</v>
       </c>
       <c r="D55" s="54" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E55" s="51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F55" s="62" t="s">
         <v>29</v>
@@ -2735,15 +2732,15 @@
       <c r="A56">
         <v>53</v>
       </c>
-      <c r="B56" s="77"/>
+      <c r="B56" s="68"/>
       <c r="C56" s="14" t="s">
         <v>88</v>
       </c>
       <c r="D56" s="54" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E56" s="51" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F56" s="62" t="s">
         <v>29</v>
@@ -2755,15 +2752,15 @@
       <c r="A57">
         <v>54</v>
       </c>
-      <c r="B57" s="77"/>
+      <c r="B57" s="68"/>
       <c r="C57" s="23" t="s">
         <v>89</v>
       </c>
       <c r="D57" s="54" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E57" s="51" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F57" s="62" t="s">
         <v>29</v>
@@ -2775,13 +2772,13 @@
       <c r="A58">
         <v>55</v>
       </c>
-      <c r="B58" s="77"/>
+      <c r="B58" s="68"/>
       <c r="C58" s="14" t="s">
         <v>90</v>
       </c>
       <c r="D58" s="54"/>
       <c r="E58" s="51" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F58" s="62" t="s">
         <v>29</v>
@@ -2793,15 +2790,15 @@
       <c r="A59">
         <v>56</v>
       </c>
-      <c r="B59" s="77"/>
+      <c r="B59" s="68"/>
       <c r="C59" s="14" t="s">
         <v>91</v>
       </c>
       <c r="D59" s="54" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E59" s="51" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F59" s="62" t="s">
         <v>29</v>
@@ -2816,7 +2813,7 @@
       <c r="A60">
         <v>57</v>
       </c>
-      <c r="B60" s="77"/>
+      <c r="B60" s="68"/>
       <c r="C60" s="14" t="s">
         <v>92</v>
       </c>
@@ -2824,7 +2821,7 @@
         <v>1</v>
       </c>
       <c r="E60" s="51" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F60" s="62" t="s">
         <v>29</v>
@@ -2839,7 +2836,7 @@
       <c r="A61">
         <v>58</v>
       </c>
-      <c r="B61" s="78" t="s">
+      <c r="B61" s="69" t="s">
         <v>93</v>
       </c>
       <c r="C61" s="14" t="s">
@@ -2849,7 +2846,7 @@
         <v>45400</v>
       </c>
       <c r="E61" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F61" s="62" t="s">
         <v>29</v>
@@ -2862,7 +2859,7 @@
       <c r="A62">
         <v>59</v>
       </c>
-      <c r="B62" s="78"/>
+      <c r="B62" s="69"/>
       <c r="C62" s="14" t="s">
         <v>95</v>
       </c>
@@ -2870,7 +2867,7 @@
         <v>45400</v>
       </c>
       <c r="E62" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F62" s="62" t="s">
         <v>29</v>
@@ -2883,15 +2880,15 @@
       <c r="A63">
         <v>60</v>
       </c>
-      <c r="B63" s="78"/>
+      <c r="B63" s="69"/>
       <c r="C63" s="14" t="s">
         <v>96</v>
       </c>
       <c r="D63" s="54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E63" s="51" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F63" s="62" t="s">
         <v>29</v>
@@ -2905,15 +2902,13 @@
       <c r="A64">
         <v>61</v>
       </c>
-      <c r="B64" s="78"/>
+      <c r="B64" s="69"/>
       <c r="C64" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D64" s="54" t="s">
-        <v>98</v>
-      </c>
+      <c r="D64" s="54"/>
       <c r="E64" s="51" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F64" s="62" t="s">
         <v>29</v>
@@ -2927,15 +2922,15 @@
       <c r="A65">
         <v>62</v>
       </c>
-      <c r="B65" s="78"/>
+      <c r="B65" s="69"/>
       <c r="C65" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D65" s="61">
         <v>45455</v>
       </c>
       <c r="E65" s="51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F65" s="62" t="s">
         <v>29</v>
@@ -2947,15 +2942,15 @@
       <c r="A66">
         <v>63</v>
       </c>
-      <c r="B66" s="78"/>
+      <c r="B66" s="69"/>
       <c r="C66" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D66" s="61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E66" s="51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F66" s="62" t="s">
         <v>29</v>
@@ -2966,13 +2961,13 @@
       <c r="A67">
         <v>64</v>
       </c>
-      <c r="B67" s="78"/>
+      <c r="B67" s="69"/>
       <c r="C67" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D67" s="61"/>
       <c r="E67" s="51" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F67" s="62" t="s">
         <v>29</v>
@@ -2983,11 +2978,11 @@
       <c r="A68">
         <v>65</v>
       </c>
-      <c r="B68" s="79" t="s">
+      <c r="B68" s="70" t="s">
+        <v>101</v>
+      </c>
+      <c r="C68" s="33" t="s">
         <v>102</v>
-      </c>
-      <c r="C68" s="33" t="s">
-        <v>103</v>
       </c>
       <c r="D68" s="39"/>
       <c r="E68" s="51" t="s">
@@ -3001,9 +2996,9 @@
       <c r="A69">
         <v>66</v>
       </c>
-      <c r="B69" s="79"/>
+      <c r="B69" s="70"/>
       <c r="C69" s="33" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D69" s="39"/>
       <c r="E69" s="1" t="s">
@@ -3017,9 +3012,9 @@
       <c r="A70">
         <v>67</v>
       </c>
-      <c r="B70" s="79"/>
+      <c r="B70" s="70"/>
       <c r="C70" s="33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D70" s="39"/>
       <c r="E70" s="1" t="s">
@@ -3031,9 +3026,9 @@
       <c r="A71">
         <v>68</v>
       </c>
-      <c r="B71" s="79"/>
+      <c r="B71" s="70"/>
       <c r="C71" s="33" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D71" s="39"/>
       <c r="E71" s="1" t="s">
@@ -3045,9 +3040,9 @@
       <c r="A72">
         <v>69</v>
       </c>
-      <c r="B72" s="80"/>
+      <c r="B72" s="71"/>
       <c r="C72" s="34" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D72" s="40"/>
       <c r="E72" s="1" t="s">
@@ -3057,16 +3052,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B20"/>
+    <mergeCell ref="B21:B25"/>
     <mergeCell ref="B26:B52"/>
     <mergeCell ref="B53:B60"/>
     <mergeCell ref="B61:B67"/>
     <mergeCell ref="B68:B72"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B20"/>
-    <mergeCell ref="B21:B25"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>
@@ -3097,10 +3092,10 @@
   <sheetData>
     <row r="1" spans="1:9" ht="14.1">
       <c r="A1" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>15</v>
@@ -3126,16 +3121,16 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B2" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D2" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E2" s="37">
         <v>15</v>
@@ -3147,7 +3142,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I2" s="37" t="s">
         <v>21</v>
@@ -3155,16 +3150,16 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E3" s="37">
         <v>15</v>
@@ -3176,7 +3171,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I3" s="37" t="s">
         <v>21</v>
@@ -3184,16 +3179,16 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B4" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E4" s="37">
         <v>15</v>
@@ -3205,7 +3200,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I4" s="37" t="s">
         <v>21</v>
@@ -3213,16 +3208,16 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B5" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E5" s="37">
         <v>15</v>
@@ -3234,7 +3229,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I5" s="37" t="s">
         <v>21</v>
@@ -3242,16 +3237,16 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B6" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E6" s="37">
         <v>15</v>
@@ -3263,7 +3258,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I6" s="37" t="s">
         <v>21</v>
@@ -3271,16 +3266,16 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="37" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B7" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E7" s="37">
         <v>15</v>
@@ -3292,7 +3287,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I7" s="37" t="s">
         <v>21</v>
@@ -3300,16 +3295,16 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B8" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E8" s="37">
         <v>30</v>
@@ -3321,7 +3316,7 @@
         <v>1</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I8" s="37" t="s">
         <v>21</v>
@@ -3329,16 +3324,16 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B9" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E9" s="37">
         <v>30</v>
@@ -3350,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I9" s="37" t="s">
         <v>21</v>
@@ -3358,16 +3353,16 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="37" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B10" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E10" s="37">
         <v>30</v>
@@ -3379,7 +3374,7 @@
         <v>1</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>21</v>
@@ -3387,16 +3382,16 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B11" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E11" s="37">
         <v>25</v>
@@ -3408,7 +3403,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I11" s="37" t="s">
         <v>21</v>
@@ -3416,16 +3411,16 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E12" s="37">
         <v>25</v>
@@ -3437,7 +3432,7 @@
         <v>1</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I12" s="37" t="s">
         <v>21</v>
@@ -3445,16 +3440,16 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B13" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E13" s="37">
         <v>30</v>
@@ -3466,7 +3461,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I13" s="37" t="s">
         <v>21</v>
@@ -3474,16 +3469,16 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B14" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E14" s="37">
         <v>30</v>
@@ -3495,7 +3490,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I14" s="37" t="s">
         <v>21</v>
@@ -3503,16 +3498,16 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B15" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E15" s="37">
         <v>30</v>
@@ -3524,7 +3519,7 @@
         <v>1</v>
       </c>
       <c r="H15" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I15" s="37" t="s">
         <v>21</v>
@@ -3532,16 +3527,16 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B16" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E16" s="37">
         <v>20</v>
@@ -3553,7 +3548,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I16" s="37" t="s">
         <v>21</v>
@@ -3561,16 +3556,16 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B17" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E17" s="37">
         <v>15</v>
@@ -3582,7 +3577,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I17" s="37" t="s">
         <v>21</v>
@@ -3590,16 +3585,16 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B18" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E18" s="37">
         <v>15</v>
@@ -3611,7 +3606,7 @@
         <v>1</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I18" s="37" t="s">
         <v>21</v>
@@ -3619,16 +3614,16 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B19" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E19" s="37">
         <v>15</v>
@@ -3640,7 +3635,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I19" s="37" t="s">
         <v>21</v>
@@ -3648,16 +3643,16 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B20" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E20" s="37">
         <v>15</v>
@@ -3669,7 +3664,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I20" s="37" t="s">
         <v>21</v>
@@ -3677,16 +3672,16 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B21" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E21" s="37">
         <v>15</v>
@@ -3698,7 +3693,7 @@
         <v>1</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I21" s="37" t="s">
         <v>21</v>

</xml_diff>